<commit_message>
QVision Registro e Inicio de Sesió de un usuario
</commit_message>
<xml_diff>
--- a/src/test/resources/data/PTP_Daniel_Valderrama27082026.xlsx
+++ b/src/test/resources/data/PTP_Daniel_Valderrama27082026.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\train\IdeaProjects\Aut-Reto-Q-Vision\src\test\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CEBF19E-D37F-49C0-A6A4-09A60EA44CAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50332369-1548-4295-BB8F-E3CE46FFC7ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="registroExitoso" sheetId="1" r:id="rId1"/>
-    <sheet name="inicioSesiónFallido-SC" sheetId="3" r:id="rId2"/>
+    <sheet name="iniciSesionExitoso" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,17 +32,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
   <si>
     <t>Contraseña</t>
   </si>
   <si>
-    <t>Mensaje de Validación</t>
-  </si>
-  <si>
-    <t>Debe ingresar su usuario y contrase&amp;ntilde;a para acceder</t>
-  </si>
-  <si>
     <t>Número de Cédula</t>
   </si>
   <si>
@@ -71,6 +65,12 @@
   </si>
   <si>
     <t>¿Desea recibir información sobre las novedades de bon-bonite en su e-mail?</t>
+  </si>
+  <si>
+    <t>¿Generar Dato Nuevo Automáticamente?</t>
+  </si>
+  <si>
+    <t>Si</t>
   </si>
 </sst>
 </file>
@@ -80,12 +80,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yyyy;@"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -134,7 +141,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -157,35 +164,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -677,7 +698,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultColWidth="9.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="16.77734375" bestFit="1" customWidth="1"/>
@@ -686,51 +707,58 @@
     <col min="4" max="4" width="29.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="65.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>12</v>
+      <c r="F1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:7">
       <c r="A2" s="2">
         <v>1000000001</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="E2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>11</v>
+      <c r="G2" s="4" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{35D20E5A-DF55-469C-95A1-77DF6A69D131}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:G2" xr:uid="{35D20E5A-DF55-469C-95A1-77DF6A69D131}">
       <formula1>"Si,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -744,20 +772,27 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B8E70CD-EB26-45CF-A29B-63062B3412EF}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" ht="57.6">
-      <c r="A2" s="3" t="s">
-        <v>2</v>
+    <row r="2" spans="1:2">
+      <c r="A2" s="2">
+        <v>1000000001</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>